<commit_message>
EPBDS-17055 Drop deprecated table types from the tutorials and examples
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example 2 - Corporate Rating/rules/Corporate Rating.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example 2 - Corporate Rating/rules/Corporate Rating.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="541">
   <si>
     <t>Domain Model</t>
   </si>
@@ -3502,6 +3502,111 @@
       </rPr>
       <t>(Double value)</t>
     </r>
+  </si>
+  <si>
+    <t>Spreadsheet Double IncreaseRiskOfOperationsScore (QualityIndicators qualityIndicators)</t>
+  </si>
+  <si>
+    <t>TerroristPersonScore</t>
+  </si>
+  <si>
+    <t>= isAnyFinOperWithTerroristPerson ? 1 : 0</t>
+  </si>
+  <si>
+    <t>PoliticianScore</t>
+  </si>
+  <si>
+    <t>= isAnyFinOperWithPolitician ? 1 : 0</t>
+  </si>
+  <si>
+    <t>CorruptCountryScore</t>
+  </si>
+  <si>
+    <t>= isAnyFinOperWithPersonFromCorruptCountry ? 1 : 0</t>
+  </si>
+  <si>
+    <t>OffshoreAccountsScore</t>
+  </si>
+  <si>
+    <t>= isAnyFinOperThroughOffshoreAccounts ? 1 : 0</t>
+  </si>
+  <si>
+    <t>ArtScore</t>
+  </si>
+  <si>
+    <t>= isAnyFinOperRelatedToArt ? 1 : 0</t>
+  </si>
+  <si>
+    <t>PreciousMetalsScore</t>
+  </si>
+  <si>
+    <t>= isAnyFinOperRelatedToPreciousMetals ? 1 : 0</t>
+  </si>
+  <si>
+    <t>NonBankInternetScore</t>
+  </si>
+  <si>
+    <t>= isAnyNonBankFinOperByInternet ? 1 : 0</t>
+  </si>
+  <si>
+    <t>= sum ( $TerroristPersonScore:$NonBankInternetScore )</t>
+  </si>
+  <si>
+    <t>= IncreaseRiskOfOperationsScoreByTotal ( $TotalScore )</t>
+  </si>
+  <si>
+    <t>SimpleRules Double IncreaseRiskOfOperationsScoreByTotal (Integer totalScore)</t>
+  </si>
+  <si>
+    <t>&gt;= 7</t>
+  </si>
+  <si>
+    <t>&gt;= 6</t>
+  </si>
+  <si>
+    <t>&gt;= 5</t>
+  </si>
+  <si>
+    <t>&gt;= 4</t>
+  </si>
+  <si>
+    <t>&gt;= 3</t>
+  </si>
+  <si>
+    <t>&gt;= 0</t>
+  </si>
+  <si>
+    <t>Spreadsheet Double IncreaseRiskOfProfileScore (QualityIndicators qualityIndicators)</t>
+  </si>
+  <si>
+    <t>ChiefOwnerScore</t>
+  </si>
+  <si>
+    <t>= isChiefAnOwnerOfAnotherCompany ? 1 : 0</t>
+  </si>
+  <si>
+    <t>FounderOwnerScore</t>
+  </si>
+  <si>
+    <t>= isFounderAnOwnerOfAnotherCompany ? 1 : 0</t>
+  </si>
+  <si>
+    <t>PoliticianBeneficiaryScore</t>
+  </si>
+  <si>
+    <t>= isBeneficiaryOwnerThePolitician ? 1 : 0</t>
+  </si>
+  <si>
+    <t>= sum ( $ChiefOwnerScore:$PoliticianBeneficiaryScore )</t>
+  </si>
+  <si>
+    <t>= IncreaseRiskOfProfileScoreByTotal ( $TotalScore )</t>
+  </si>
+  <si>
+    <t>SimpleRules Double IncreaseRiskOfProfileScoreByTotal (Integer totalScore)</t>
+  </si>
+  <si>
+    <t>Increase Risk of Profile Score</t>
   </si>
 </sst>
 </file>
@@ -9148,11 +9253,11 @@
   <sheetPr>
     <tabColor theme="0" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="B1:K55"/>
+  <dimension ref="B1:K61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="25.54296875" customWidth="1"/>
-    <col min="4" max="4" width="22.08984375" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.08984375" bestFit="1" customWidth="1"/>
   </cols>
@@ -9645,181 +9750,135 @@
     </row>
     <row r="40" spans="2:10" ht="16.2" x14ac:dyDescent="0.35">
       <c r="B40" s="10"/>
-      <c r="C40" s="133" t="s">
-        <v>479</v>
-      </c>
-      <c r="D40" s="133"/>
-      <c r="E40" s="133"/>
-      <c r="F40" s="133"/>
-      <c r="G40" s="133"/>
-      <c r="H40" s="133"/>
-      <c r="I40" s="133"/>
+      <c r="C40" s="124" t="s">
+        <v>530</v>
+      </c>
+      <c r="D40" s="124"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
       <c r="J40" s="10"/>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B41" s="10"/>
-      <c r="C41" s="76" t="s">
-        <v>235</v>
-      </c>
-      <c r="D41" s="76" t="s">
-        <v>236</v>
-      </c>
-      <c r="E41" s="76" t="s">
-        <v>237</v>
-      </c>
-      <c r="F41" s="143" t="s">
-        <v>238</v>
-      </c>
-      <c r="G41" s="143"/>
-      <c r="H41" s="143"/>
-      <c r="I41" s="143"/>
+      <c r="C41" s="120" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
       <c r="J41" s="10"/>
     </row>
-    <row r="42" spans="2:10" ht="28.2" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B42" s="10"/>
-      <c r="C42" s="81" t="s">
-        <v>246</v>
-      </c>
-      <c r="D42" s="76" t="s">
-        <v>236</v>
-      </c>
-      <c r="E42" s="84" t="s">
-        <v>237</v>
-      </c>
-      <c r="F42" s="144" t="s">
-        <v>247</v>
-      </c>
-      <c r="G42" s="144"/>
-      <c r="H42" s="144"/>
-      <c r="I42" s="144"/>
+      <c r="C42" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="D42" s="154" t="s">
+        <v>532</v>
+      </c>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="10"/>
       <c r="J42" s="10"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B43" s="10"/>
-      <c r="C43" s="76" t="s">
-        <v>239</v>
-      </c>
-      <c r="D43" s="85"/>
-      <c r="E43" s="84"/>
-      <c r="F43" s="88">
-        <v>3</v>
-      </c>
-      <c r="G43" s="89">
-        <v>2</v>
-      </c>
-      <c r="H43" s="93" t="s">
-        <v>244</v>
-      </c>
-      <c r="I43" s="90">
-        <v>1</v>
-      </c>
+      <c r="C43" s="5" t="s">
+        <v>533</v>
+      </c>
+      <c r="D43" s="154" t="s">
+        <v>534</v>
+      </c>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
       <c r="J43" s="10"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B44" s="10"/>
-      <c r="C44" s="76" t="s">
-        <v>241</v>
-      </c>
-      <c r="D44" s="84" t="s">
-        <v>242</v>
-      </c>
-      <c r="E44" s="84"/>
-      <c r="F44" s="91">
-        <v>3</v>
-      </c>
-      <c r="G44" s="78">
-        <v>2</v>
-      </c>
-      <c r="H44" s="78">
-        <v>1</v>
-      </c>
-      <c r="I44" s="92">
-        <v>0</v>
-      </c>
+      <c r="C44" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="D44" s="154" t="s">
+        <v>536</v>
+      </c>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10"/>
       <c r="J44" s="10"/>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B45" s="10"/>
-      <c r="C45" s="76" t="s">
-        <v>229</v>
-      </c>
-      <c r="D45" s="85"/>
-      <c r="E45" s="44"/>
-      <c r="F45" s="55">
-        <v>1</v>
-      </c>
-      <c r="G45" s="55">
-        <v>0</v>
-      </c>
-      <c r="H45" s="55">
-        <v>0</v>
-      </c>
-      <c r="I45" s="55">
-        <v>0</v>
-      </c>
+      <c r="C45" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="D45" s="154" t="s">
+        <v>537</v>
+      </c>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
       <c r="J45" s="10"/>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B46" s="10"/>
-      <c r="C46" s="58" t="s">
-        <v>376</v>
-      </c>
-      <c r="D46" s="84" t="s">
-        <v>243</v>
-      </c>
-      <c r="E46" s="44">
-        <v>1</v>
-      </c>
-      <c r="F46" s="58" t="s">
-        <v>11</v>
-      </c>
-      <c r="G46" s="55"/>
-      <c r="H46" s="55"/>
-      <c r="I46" s="55"/>
+      <c r="C46" s="156" t="s">
+        <v>229</v>
+      </c>
+      <c r="D46" s="157" t="s">
+        <v>538</v>
+      </c>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="10"/>
       <c r="J46" s="10"/>
     </row>
-    <row r="47" spans="2:10" ht="28.2" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B47" s="10"/>
-      <c r="C47" s="86" t="s">
-        <v>377</v>
-      </c>
-      <c r="D47" s="84" t="s">
-        <v>243</v>
-      </c>
-      <c r="E47" s="44">
-        <v>1</v>
-      </c>
-      <c r="F47" s="86" t="s">
-        <v>11</v>
-      </c>
-      <c r="G47" s="55"/>
-      <c r="H47" s="55"/>
-      <c r="I47" s="55"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="10"/>
       <c r="J47" s="10"/>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B48" s="10"/>
-      <c r="C48" s="58" t="s">
-        <v>39</v>
-      </c>
-      <c r="D48" s="87" t="s">
-        <v>243</v>
-      </c>
-      <c r="E48" s="44">
-        <v>1</v>
-      </c>
-      <c r="F48" s="58" t="s">
-        <v>11</v>
-      </c>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="10"/>
       <c r="J48" s="10"/>
     </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:10" ht="16.2" x14ac:dyDescent="0.35">
       <c r="B49" s="10"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
+      <c r="C49" s="133" t="s">
+        <v>539</v>
+      </c>
+      <c r="D49" s="134"/>
       <c r="E49" s="10"/>
       <c r="F49" s="10"/>
       <c r="G49" s="10"/>
@@ -9829,8 +9888,12 @@
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
+      <c r="C50" s="81" t="s">
+        <v>241</v>
+      </c>
+      <c r="D50" s="50" t="s">
+        <v>540</v>
+      </c>
       <c r="E50" s="10"/>
       <c r="F50" s="10"/>
       <c r="G50" s="10"/>
@@ -9838,12 +9901,14 @@
       <c r="I50" s="10"/>
       <c r="J50" s="10"/>
     </row>
-    <row r="51" spans="2:10" ht="16.2" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B51" s="10"/>
-      <c r="C51" s="133" t="s">
-        <v>480</v>
-      </c>
-      <c r="D51" s="134"/>
+      <c r="C51" s="44" t="s">
+        <v>528</v>
+      </c>
+      <c r="D51" s="82">
+        <v>3</v>
+      </c>
       <c r="E51" s="10"/>
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
@@ -9853,11 +9918,11 @@
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B52" s="10"/>
-      <c r="C52" s="81" t="s">
-        <v>251</v>
-      </c>
-      <c r="D52" s="50" t="s">
-        <v>250</v>
+      <c r="C52" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="D52" s="82">
+        <v>2</v>
       </c>
       <c r="E52" s="10"/>
       <c r="F52" s="10"/>
@@ -9869,10 +9934,10 @@
     <row r="53" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B53" s="10"/>
       <c r="C53" s="44" t="s">
-        <v>18</v>
-      </c>
-      <c r="D53" s="96" t="s">
-        <v>252</v>
+        <v>140</v>
+      </c>
+      <c r="D53" s="82">
+        <v>1.5</v>
       </c>
       <c r="E53" s="10"/>
       <c r="F53" s="10"/>
@@ -9884,7 +9949,7 @@
     <row r="54" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B54" s="10"/>
       <c r="C54" s="58" t="s">
-        <v>19</v>
+        <v>529</v>
       </c>
       <c r="D54" s="80">
         <v>1</v>
@@ -9907,8 +9972,88 @@
       <c r="I55" s="10"/>
       <c r="J55" s="10"/>
     </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B56" s="10"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="10"/>
+      <c r="E56" s="10"/>
+      <c r="F56" s="10"/>
+      <c r="G56" s="10"/>
+      <c r="H56" s="10"/>
+      <c r="I56" s="10"/>
+      <c r="J56" s="10"/>
+    </row>
+    <row r="57" spans="2:10" ht="16.2" x14ac:dyDescent="0.35">
+      <c r="B57" s="10"/>
+      <c r="C57" s="133" t="s">
+        <v>480</v>
+      </c>
+      <c r="D57" s="134"/>
+      <c r="E57" s="10"/>
+      <c r="F57" s="10"/>
+      <c r="G57" s="10"/>
+      <c r="H57" s="10"/>
+      <c r="I57" s="10"/>
+      <c r="J57" s="10"/>
+    </row>
+    <row r="58" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B58" s="10"/>
+      <c r="C58" s="81" t="s">
+        <v>251</v>
+      </c>
+      <c r="D58" s="50" t="s">
+        <v>250</v>
+      </c>
+      <c r="E58" s="10"/>
+      <c r="F58" s="10"/>
+      <c r="G58" s="10"/>
+      <c r="H58" s="10"/>
+      <c r="I58" s="10"/>
+      <c r="J58" s="10"/>
+    </row>
+    <row r="59" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B59" s="10"/>
+      <c r="C59" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="D59" s="96" t="s">
+        <v>252</v>
+      </c>
+      <c r="E59" s="10"/>
+      <c r="F59" s="10"/>
+      <c r="G59" s="10"/>
+      <c r="H59" s="10"/>
+      <c r="I59" s="10"/>
+      <c r="J59" s="10"/>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B60" s="10"/>
+      <c r="C60" s="58" t="s">
+        <v>19</v>
+      </c>
+      <c r="D60" s="80">
+        <v>1</v>
+      </c>
+      <c r="E60" s="10"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="10"/>
+      <c r="H60" s="10"/>
+      <c r="I60" s="10"/>
+      <c r="J60" s="10"/>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="10"/>
+      <c r="E61" s="10"/>
+      <c r="F61" s="10"/>
+      <c r="G61" s="10"/>
+      <c r="H61" s="10"/>
+      <c r="I61" s="10"/>
+      <c r="J61" s="10"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="F18:F23"/>
@@ -9918,11 +10063,10 @@
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C16:F16"/>
     <mergeCell ref="D10:D12"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C57:D57"/>
     <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C40:I40"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C49:D49"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="K1" location="'Rating Algorithm'!A48" display="'Rating Algorithm'!A48" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
@@ -10175,11 +10319,11 @@
   <sheetPr>
     <tabColor theme="0" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="B1:O48"/>
+  <dimension ref="B1:O58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="29.54296875" customWidth="1"/>
-    <col min="4" max="4" width="25.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
     <col min="6" max="6" width="6.54296875" customWidth="1"/>
     <col min="8" max="8" width="7.453125" customWidth="1"/>
   </cols>
@@ -10595,333 +10739,247 @@
     </row>
     <row r="28" spans="2:14" ht="16.2" x14ac:dyDescent="0.35">
       <c r="B28" s="10"/>
-      <c r="C28" s="133" t="s">
-        <v>484</v>
-      </c>
-      <c r="D28" s="133"/>
-      <c r="E28" s="133"/>
-      <c r="F28" s="133"/>
-      <c r="G28" s="133"/>
-      <c r="H28" s="133"/>
-      <c r="I28" s="133"/>
-      <c r="J28" s="133"/>
-      <c r="K28" s="133"/>
-      <c r="L28" s="133"/>
-      <c r="M28" s="133"/>
+      <c r="C28" s="124" t="s">
+        <v>506</v>
+      </c>
+      <c r="D28" s="124"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
       <c r="N28" s="10"/>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B29" s="10"/>
-      <c r="C29" s="76" t="s">
-        <v>235</v>
-      </c>
-      <c r="D29" s="76" t="s">
-        <v>236</v>
-      </c>
-      <c r="E29" s="76" t="s">
-        <v>237</v>
-      </c>
-      <c r="F29" s="143" t="s">
-        <v>238</v>
-      </c>
-      <c r="G29" s="143"/>
-      <c r="H29" s="143"/>
-      <c r="I29" s="143"/>
-      <c r="J29" s="143"/>
-      <c r="K29" s="143"/>
-      <c r="L29" s="143"/>
-      <c r="M29" s="143"/>
+      <c r="C29" s="120" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
       <c r="N29" s="10"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B30" s="10"/>
-      <c r="C30" s="81" t="s">
-        <v>294</v>
-      </c>
-      <c r="D30" s="76" t="s">
-        <v>236</v>
-      </c>
-      <c r="E30" s="84" t="s">
-        <v>237</v>
-      </c>
-      <c r="F30" s="144" t="s">
-        <v>295</v>
-      </c>
-      <c r="G30" s="144"/>
-      <c r="H30" s="144"/>
-      <c r="I30" s="144"/>
-      <c r="J30" s="144"/>
-      <c r="K30" s="144"/>
-      <c r="L30" s="144"/>
-      <c r="M30" s="144"/>
+      <c r="C30" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="D30" s="154" t="s">
+        <v>508</v>
+      </c>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
       <c r="N30" s="10"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B31" s="10"/>
-      <c r="C31" s="76" t="s">
-        <v>239</v>
-      </c>
-      <c r="D31" s="85"/>
-      <c r="E31" s="84"/>
-      <c r="F31" s="98" t="s">
-        <v>296</v>
-      </c>
-      <c r="G31" s="99">
-        <v>4</v>
-      </c>
-      <c r="H31" s="93" t="s">
-        <v>297</v>
-      </c>
-      <c r="I31" s="90">
-        <v>3</v>
-      </c>
-      <c r="J31" s="100" t="s">
-        <v>298</v>
-      </c>
-      <c r="K31" s="90">
-        <v>2</v>
-      </c>
-      <c r="L31" s="100" t="s">
-        <v>244</v>
-      </c>
-      <c r="M31" s="90">
-        <v>1</v>
-      </c>
+      <c r="C31" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="D31" s="154" t="s">
+        <v>510</v>
+      </c>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
       <c r="N31" s="10"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B32" s="10"/>
-      <c r="C32" s="76" t="s">
-        <v>241</v>
-      </c>
-      <c r="D32" s="84" t="s">
-        <v>242</v>
-      </c>
-      <c r="E32" s="84"/>
-      <c r="F32" s="91">
-        <v>7</v>
-      </c>
-      <c r="G32" s="78">
-        <v>6</v>
-      </c>
-      <c r="H32" s="78">
-        <v>5</v>
-      </c>
-      <c r="I32" s="92">
-        <v>4</v>
-      </c>
-      <c r="J32" s="92">
-        <v>3</v>
-      </c>
-      <c r="K32" s="92">
-        <v>2</v>
-      </c>
-      <c r="L32" s="92">
-        <v>1</v>
-      </c>
-      <c r="M32" s="92">
-        <v>0</v>
-      </c>
+      <c r="C32" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="D32" s="154" t="s">
+        <v>512</v>
+      </c>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
+      <c r="L32" s="10"/>
+      <c r="M32" s="10"/>
       <c r="N32" s="10"/>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B33" s="10"/>
-      <c r="C33" s="76" t="s">
-        <v>229</v>
-      </c>
-      <c r="D33" s="85"/>
-      <c r="E33" s="44"/>
-      <c r="F33" s="55">
-        <v>1</v>
-      </c>
-      <c r="G33" s="55">
-        <v>0</v>
-      </c>
-      <c r="H33" s="55">
-        <v>0</v>
-      </c>
-      <c r="I33" s="55">
-        <v>0</v>
-      </c>
-      <c r="J33" s="55">
-        <v>0</v>
-      </c>
-      <c r="K33" s="55">
-        <v>0</v>
-      </c>
-      <c r="L33" s="55">
-        <v>0</v>
-      </c>
-      <c r="M33" s="55">
-        <v>0</v>
-      </c>
+      <c r="C33" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="D33" s="154" t="s">
+        <v>514</v>
+      </c>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="10"/>
+      <c r="M33" s="10"/>
       <c r="N33" s="10"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B34" s="10"/>
-      <c r="C34" s="58" t="s">
-        <v>52</v>
-      </c>
-      <c r="D34" s="84" t="s">
-        <v>243</v>
-      </c>
-      <c r="E34" s="44">
-        <v>1</v>
-      </c>
-      <c r="F34" s="58" t="s">
-        <v>11</v>
-      </c>
-      <c r="G34" s="55"/>
-      <c r="H34" s="55"/>
-      <c r="I34" s="55"/>
-      <c r="J34" s="55"/>
-      <c r="K34" s="55"/>
-      <c r="L34" s="55"/>
-      <c r="M34" s="55"/>
+      <c r="C34" s="5" t="s">
+        <v>515</v>
+      </c>
+      <c r="D34" s="154" t="s">
+        <v>516</v>
+      </c>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
       <c r="N34" s="10"/>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B35" s="10"/>
-      <c r="C35" s="86" t="s">
-        <v>53</v>
-      </c>
-      <c r="D35" s="84" t="s">
-        <v>243</v>
-      </c>
-      <c r="E35" s="44">
-        <v>1</v>
-      </c>
-      <c r="F35" s="86" t="s">
-        <v>11</v>
-      </c>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
-      <c r="I35" s="55"/>
-      <c r="J35" s="55"/>
-      <c r="K35" s="55"/>
-      <c r="L35" s="55"/>
-      <c r="M35" s="55"/>
+      <c r="C35" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="D35" s="154" t="s">
+        <v>518</v>
+      </c>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
+      <c r="K35" s="10"/>
+      <c r="L35" s="10"/>
+      <c r="M35" s="10"/>
       <c r="N35" s="10"/>
     </row>
-    <row r="36" spans="2:14" ht="28.2" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B36" s="10"/>
-      <c r="C36" s="58" t="s">
-        <v>54</v>
-      </c>
-      <c r="D36" s="84" t="s">
-        <v>243</v>
-      </c>
-      <c r="E36" s="44">
-        <v>1</v>
-      </c>
-      <c r="F36" s="86" t="s">
-        <v>11</v>
-      </c>
-      <c r="G36" s="55"/>
-      <c r="H36" s="55"/>
-      <c r="I36" s="55"/>
-      <c r="J36" s="55"/>
-      <c r="K36" s="55"/>
-      <c r="L36" s="55"/>
-      <c r="M36" s="55"/>
+      <c r="C36" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="D36" s="154" t="s">
+        <v>520</v>
+      </c>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="10"/>
+      <c r="L36" s="10"/>
+      <c r="M36" s="10"/>
       <c r="N36" s="10"/>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B37" s="10"/>
-      <c r="C37" s="58" t="s">
-        <v>55</v>
-      </c>
-      <c r="D37" s="84" t="s">
-        <v>243</v>
-      </c>
-      <c r="E37" s="44">
-        <v>1</v>
-      </c>
-      <c r="F37" s="86" t="s">
-        <v>11</v>
-      </c>
-      <c r="G37" s="55"/>
-      <c r="H37" s="55"/>
-      <c r="I37" s="55"/>
-      <c r="J37" s="55"/>
-      <c r="K37" s="55"/>
-      <c r="L37" s="55"/>
-      <c r="M37" s="55"/>
+      <c r="C37" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="D37" s="154" t="s">
+        <v>521</v>
+      </c>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
       <c r="N37" s="10"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B38" s="10"/>
-      <c r="C38" s="58" t="s">
-        <v>56</v>
-      </c>
-      <c r="D38" s="84" t="s">
-        <v>243</v>
-      </c>
-      <c r="E38" s="44">
-        <v>1</v>
-      </c>
-      <c r="F38" s="86" t="s">
-        <v>11</v>
-      </c>
-      <c r="G38" s="55"/>
-      <c r="H38" s="55"/>
-      <c r="I38" s="55"/>
-      <c r="J38" s="55"/>
-      <c r="K38" s="55"/>
-      <c r="L38" s="55"/>
-      <c r="M38" s="55"/>
+      <c r="C38" s="156" t="s">
+        <v>229</v>
+      </c>
+      <c r="D38" s="157" t="s">
+        <v>522</v>
+      </c>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10"/>
       <c r="N38" s="10"/>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B39" s="10"/>
-      <c r="C39" s="58" t="s">
-        <v>57</v>
-      </c>
-      <c r="D39" s="84" t="s">
-        <v>243</v>
-      </c>
-      <c r="E39" s="44">
-        <v>1</v>
-      </c>
-      <c r="F39" s="86" t="s">
-        <v>11</v>
-      </c>
-      <c r="G39" s="55"/>
-      <c r="H39" s="55"/>
-      <c r="I39" s="55"/>
-      <c r="J39" s="55"/>
-      <c r="K39" s="55"/>
-      <c r="L39" s="55"/>
-      <c r="M39" s="55"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+      <c r="M39" s="10"/>
       <c r="N39" s="10"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B40" s="10"/>
-      <c r="C40" s="58" t="s">
-        <v>58</v>
-      </c>
-      <c r="D40" s="87" t="s">
-        <v>243</v>
-      </c>
-      <c r="E40" s="44">
-        <v>1</v>
-      </c>
-      <c r="F40" s="58" t="s">
-        <v>11</v>
-      </c>
-      <c r="G40" s="55"/>
-      <c r="H40" s="55"/>
-      <c r="I40" s="55"/>
-      <c r="J40" s="55"/>
-      <c r="K40" s="55"/>
-      <c r="L40" s="55"/>
-      <c r="M40" s="55"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
       <c r="N40" s="10"/>
     </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:14" ht="16.2" x14ac:dyDescent="0.35">
       <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
+      <c r="C41" s="133" t="s">
+        <v>523</v>
+      </c>
+      <c r="D41" s="134"/>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
       <c r="G41" s="10"/>
@@ -10935,8 +10993,12 @@
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
+      <c r="C42" s="81" t="s">
+        <v>241</v>
+      </c>
+      <c r="D42" s="50" t="s">
+        <v>299</v>
+      </c>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
@@ -10948,13 +11010,15 @@
       <c r="M42" s="10"/>
       <c r="N42" s="10"/>
     </row>
-    <row r="43" spans="2:14" ht="16.2" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B43" s="10"/>
-      <c r="C43" s="133" t="s">
-        <v>485</v>
-      </c>
-      <c r="D43" s="133"/>
-      <c r="E43" s="133"/>
+      <c r="C43" s="44" t="s">
+        <v>524</v>
+      </c>
+      <c r="D43" s="82">
+        <v>4.5</v>
+      </c>
+      <c r="E43" s="10"/>
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
       <c r="H43" s="10"/>
@@ -10967,15 +11031,13 @@
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B44" s="10"/>
-      <c r="C44" s="49" t="s">
-        <v>300</v>
-      </c>
-      <c r="D44" s="49" t="s">
-        <v>301</v>
-      </c>
-      <c r="E44" s="50" t="s">
-        <v>229</v>
-      </c>
+      <c r="C44" s="44" t="s">
+        <v>525</v>
+      </c>
+      <c r="D44" s="82">
+        <v>4</v>
+      </c>
+      <c r="E44" s="10"/>
       <c r="F44" s="10"/>
       <c r="G44" s="10"/>
       <c r="H44" s="10"/>
@@ -10989,12 +11051,12 @@
     <row r="45" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B45" s="10"/>
       <c r="C45" s="44" t="s">
-        <v>11</v>
-      </c>
-      <c r="D45" s="44"/>
-      <c r="E45" s="145" t="s">
-        <v>252</v>
-      </c>
+        <v>526</v>
+      </c>
+      <c r="D45" s="82">
+        <v>3.5</v>
+      </c>
+      <c r="E45" s="10"/>
       <c r="F45" s="10"/>
       <c r="G45" s="10"/>
       <c r="H45" s="10"/>
@@ -11007,11 +11069,13 @@
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B46" s="10"/>
-      <c r="C46" s="44"/>
-      <c r="D46" s="44" t="s">
-        <v>11</v>
-      </c>
-      <c r="E46" s="146"/>
+      <c r="C46" s="44" t="s">
+        <v>527</v>
+      </c>
+      <c r="D46" s="82">
+        <v>3</v>
+      </c>
+      <c r="E46" s="10"/>
       <c r="F46" s="10"/>
       <c r="G46" s="10"/>
       <c r="H46" s="10"/>
@@ -11024,11 +11088,13 @@
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B47" s="10"/>
-      <c r="C47" s="86"/>
-      <c r="D47" s="86"/>
-      <c r="E47" s="101">
-        <v>1</v>
-      </c>
+      <c r="C47" s="44" t="s">
+        <v>528</v>
+      </c>
+      <c r="D47" s="82">
+        <v>2.5</v>
+      </c>
+      <c r="E47" s="10"/>
       <c r="F47" s="10"/>
       <c r="G47" s="10"/>
       <c r="H47" s="10"/>
@@ -11041,8 +11107,12 @@
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
+      <c r="C48" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="D48" s="82">
+        <v>2</v>
+      </c>
       <c r="E48" s="10"/>
       <c r="F48" s="10"/>
       <c r="G48" s="10"/>
@@ -11054,17 +11124,190 @@
       <c r="M48" s="10"/>
       <c r="N48" s="10"/>
     </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B49" s="10"/>
+      <c r="C49" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="D49" s="82">
+        <v>1.5</v>
+      </c>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
+      <c r="J49" s="10"/>
+      <c r="K49" s="10"/>
+      <c r="L49" s="10"/>
+      <c r="M49" s="10"/>
+      <c r="N49" s="10"/>
+    </row>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B50" s="10"/>
+      <c r="C50" s="58" t="s">
+        <v>529</v>
+      </c>
+      <c r="D50" s="80">
+        <v>1</v>
+      </c>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="10"/>
+      <c r="J50" s="10"/>
+      <c r="K50" s="10"/>
+      <c r="L50" s="10"/>
+      <c r="M50" s="10"/>
+      <c r="N50" s="10"/>
+    </row>
+    <row r="51" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10"/>
+      <c r="I51" s="10"/>
+      <c r="J51" s="10"/>
+      <c r="K51" s="10"/>
+      <c r="L51" s="10"/>
+      <c r="M51" s="10"/>
+      <c r="N51" s="10"/>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="10"/>
+      <c r="G52" s="10"/>
+      <c r="H52" s="10"/>
+      <c r="I52" s="10"/>
+      <c r="J52" s="10"/>
+      <c r="K52" s="10"/>
+      <c r="L52" s="10"/>
+      <c r="M52" s="10"/>
+      <c r="N52" s="10"/>
+    </row>
+    <row r="53" spans="2:14" ht="16.2" x14ac:dyDescent="0.35">
+      <c r="B53" s="10"/>
+      <c r="C53" s="133" t="s">
+        <v>485</v>
+      </c>
+      <c r="D53" s="133"/>
+      <c r="E53" s="133"/>
+      <c r="F53" s="10"/>
+      <c r="G53" s="10"/>
+      <c r="H53" s="10"/>
+      <c r="I53" s="10"/>
+      <c r="J53" s="10"/>
+      <c r="K53" s="10"/>
+      <c r="L53" s="10"/>
+      <c r="M53" s="10"/>
+      <c r="N53" s="10"/>
+    </row>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B54" s="10"/>
+      <c r="C54" s="49" t="s">
+        <v>300</v>
+      </c>
+      <c r="D54" s="49" t="s">
+        <v>301</v>
+      </c>
+      <c r="E54" s="50" t="s">
+        <v>229</v>
+      </c>
+      <c r="F54" s="10"/>
+      <c r="G54" s="10"/>
+      <c r="H54" s="10"/>
+      <c r="I54" s="10"/>
+      <c r="J54" s="10"/>
+      <c r="K54" s="10"/>
+      <c r="L54" s="10"/>
+      <c r="M54" s="10"/>
+      <c r="N54" s="10"/>
+    </row>
+    <row r="55" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B55" s="10"/>
+      <c r="C55" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="D55" s="44"/>
+      <c r="E55" s="145" t="s">
+        <v>252</v>
+      </c>
+      <c r="F55" s="10"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="10"/>
+      <c r="I55" s="10"/>
+      <c r="J55" s="10"/>
+      <c r="K55" s="10"/>
+      <c r="L55" s="10"/>
+      <c r="M55" s="10"/>
+      <c r="N55" s="10"/>
+    </row>
+    <row r="56" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B56" s="10"/>
+      <c r="C56" s="44"/>
+      <c r="D56" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" s="146"/>
+      <c r="F56" s="10"/>
+      <c r="G56" s="10"/>
+      <c r="H56" s="10"/>
+      <c r="I56" s="10"/>
+      <c r="J56" s="10"/>
+      <c r="K56" s="10"/>
+      <c r="L56" s="10"/>
+      <c r="M56" s="10"/>
+      <c r="N56" s="10"/>
+    </row>
+    <row r="57" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B57" s="10"/>
+      <c r="C57" s="86"/>
+      <c r="D57" s="86"/>
+      <c r="E57" s="101">
+        <v>1</v>
+      </c>
+      <c r="F57" s="10"/>
+      <c r="G57" s="10"/>
+      <c r="H57" s="10"/>
+      <c r="I57" s="10"/>
+      <c r="J57" s="10"/>
+      <c r="K57" s="10"/>
+      <c r="L57" s="10"/>
+      <c r="M57" s="10"/>
+      <c r="N57" s="10"/>
+    </row>
+    <row r="58" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B58" s="10"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="10"/>
+      <c r="E58" s="10"/>
+      <c r="F58" s="10"/>
+      <c r="G58" s="10"/>
+      <c r="H58" s="10"/>
+      <c r="I58" s="10"/>
+      <c r="J58" s="10"/>
+      <c r="K58" s="10"/>
+      <c r="L58" s="10"/>
+      <c r="M58" s="10"/>
+      <c r="N58" s="10"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="E45:E46"/>
+  <mergeCells count="8">
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="E55:E56"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F30:M30"/>
-    <mergeCell ref="F29:M29"/>
-    <mergeCell ref="C28:M28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C41:D41"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O1" location="'Rating Algorithm'!A66" display="'Rating Algorithm'!A66" xr:uid="{00000000-0004-0000-0500-000000000000}"/>

</xml_diff>